<commit_message>
Generating Timetable for 2023-24
</commit_message>
<xml_diff>
--- a/backend/output_db/final_timetable.xlsx
+++ b/backend/output_db/final_timetable.xlsx
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,49 +431,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Slot 1</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Slot 2</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Slot 3</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Slot 5</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Slot 6</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Slot 7</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Slot 8</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
@@ -513,7 +525,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
@@ -565,7 +577,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
@@ -607,7 +619,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -659,7 +671,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
@@ -720,49 +732,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Slot 1</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Slot 2</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Slot 3</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Slot 5</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Slot 6</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Slot 7</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Slot 8</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
@@ -820,7 +832,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
@@ -874,7 +886,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
@@ -924,7 +936,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -977,7 +989,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>
@@ -1043,49 +1055,49 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Slot 1</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Slot 2</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Slot 3</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Slot 5</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Slot 6</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Slot 7</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Slot 8</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
@@ -1130,7 +1142,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
@@ -1177,7 +1189,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
@@ -1224,7 +1236,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -1274,7 +1286,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>

</xml_diff>